<commit_message>
Add consultation tracker with Fukushima Yui and Aoi-san records
- New consultation_tracker.py module with Excel export (openpyxl)
- consultations.json with 2 records: 福島由衣 (high school student) and 蒼井さん (film professional)
- Updated run.py to add menu item 6 for consultation tracker
- Excel includes color-coded group headers, alternating rows, freeze panes

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019hSGnxN1pjVQgYvqknyZZA
</commit_message>
<xml_diff>
--- a/consultation_tracker.xlsx
+++ b/consultation_tracker.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,11 @@
         <fgColor rgb="002F5496"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -118,6 +123,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -485,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:X4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -767,6 +778,126 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>蒼井さん</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>映画・メディア研究の大学院進学（2028年）。将来PhD取得→海外映画・メディア企業または研究職。</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>オランダ（リサーチマスター第一志望）。映画学校（映画美学校・渋谷）2026年9月入学予定。</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-21（映画美学校入学申し込み締め切り＝IELTSスコア取得の実質デッドライン）</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>6.0（推定）</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>2026-05末（初受験）</t>
+        </is>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t>2026-08（7日・10日・17〜18日の3回予約済み）</t>
+        </is>
+      </c>
+      <c r="T4" s="10" t="inlineStr">
+        <is>
+          <t>独学（2月〜）。平日3〜4時間・土日11時間可能。毎日：パート1をAIランダム出題→採点→音読、パート2ネタ準備・音読、瞬間英作文20問。休日：パート3練習追加。ガバ（オンライン英会話）週1。</t>
+        </is>
+      </c>
+      <c r="U4" s="10" t="inlineStr">
+        <is>
+          <t>スピーキング（5.0）が最大課題。暗記型のアプローチになっており、パート3で質問とずれた回答をしてしまった。瞬間英作文は試験との親和性が低い可能性あり。ライティング6.5の再現性に自信なし（AIだと5.5評価）。</t>
+        </is>
+      </c>
+      <c r="V4" s="10" t="inlineStr">
+        <is>
+          <t>「スピーキングをどう伸ばせばいいかわからない」「暗記してバレたのか不安」「映画学校が始まったら勉強時間がなくなる」「コーチング費用と映画学校費用・大学院費用が重なる」「8月に取れなければ映画学校入学を諦めることも覚悟している」</t>
+        </is>
+      </c>
+      <c r="W4" s="10" t="inlineStr">
+        <is>
+          <t>〜8/21：IELTS集中（8月に3回受験）。8/21までにスコア取得で映画美学校入学確定。9月〜：映画美学校（週2夜＋土日）通学開始→並行学習は現実的でないと判断。2028年：海外大学院（オランダ）進学目標。</t>
+        </is>
+      </c>
+      <c r="X4" s="10" t="inlineStr">
+        <is>
+          <t>Instagram経由で4月登録。職歴：広告代理店4年（映像プランナー）→東映アニメーション（テーマパーク宣伝、海外4割の部署）。大学：教育学部複合文化学科（映像・映画研究）。留学経験：ボストン半年（語学学校）。日本の大学院科目履修生も検討中。スピーキングコーチング（3ヶ月・2000ポンド≈40万）を提案、翌日18時までに返事予定。お金面では迷いあるが内容には前向き。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:G1"/>

</xml_diff>